<commit_message>
fix(ai): future covariates sincos transform. wrong period of pembagian_waktu/hari and hari_per_minggu
</commit_message>
<xml_diff>
--- a/reports/nbeats_future_prediction_results.xlsx
+++ b/reports/nbeats_future_prediction_results.xlsx
@@ -471,19 +471,19 @@
         <v>45839</v>
       </c>
       <c r="B2" t="n">
-        <v>21.28914642333984</v>
+        <v>13.66680908203125</v>
       </c>
       <c r="C2" t="n">
-        <v>22.74205017089844</v>
+        <v>22.34885215759277</v>
       </c>
       <c r="D2" t="n">
-        <v>643.2750244140625</v>
+        <v>493.5171203613281</v>
       </c>
       <c r="E2" t="n">
-        <v>25.90433120727539</v>
+        <v>18.31430816650391</v>
       </c>
       <c r="F2" t="n">
-        <v>11.3208646774292</v>
+        <v>11.27921772003174</v>
       </c>
     </row>
     <row r="3">
@@ -491,19 +491,19 @@
         <v>45839.04166666666</v>
       </c>
       <c r="B3" t="n">
-        <v>17.26388740539551</v>
+        <v>15.72303199768066</v>
       </c>
       <c r="C3" t="n">
-        <v>21.13069725036621</v>
+        <v>21.53035163879395</v>
       </c>
       <c r="D3" t="n">
-        <v>734.884033203125</v>
+        <v>480.7809143066406</v>
       </c>
       <c r="E3" t="n">
-        <v>17.34470748901367</v>
+        <v>17.98626136779785</v>
       </c>
       <c r="F3" t="n">
-        <v>13.07268142700195</v>
+        <v>10.31490135192871</v>
       </c>
     </row>
     <row r="4">
@@ -511,19 +511,19 @@
         <v>45839.08333333334</v>
       </c>
       <c r="B4" t="n">
-        <v>20.79070663452148</v>
+        <v>13.92644500732422</v>
       </c>
       <c r="C4" t="n">
-        <v>29.03361129760742</v>
+        <v>20.73153495788574</v>
       </c>
       <c r="D4" t="n">
-        <v>764.6969604492188</v>
+        <v>393.5574951171875</v>
       </c>
       <c r="E4" t="n">
-        <v>23.04388427734375</v>
+        <v>22.21829223632812</v>
       </c>
       <c r="F4" t="n">
-        <v>9.320321083068848</v>
+        <v>6.941885948181152</v>
       </c>
     </row>
     <row r="5">
@@ -531,19 +531,19 @@
         <v>45839.125</v>
       </c>
       <c r="B5" t="n">
-        <v>17.59259223937988</v>
+        <v>19.11257553100586</v>
       </c>
       <c r="C5" t="n">
-        <v>23.69670295715332</v>
+        <v>28.15279197692871</v>
       </c>
       <c r="D5" t="n">
-        <v>456.4663391113281</v>
+        <v>570.4630126953125</v>
       </c>
       <c r="E5" t="n">
-        <v>18.03978157043457</v>
+        <v>21.31902503967285</v>
       </c>
       <c r="F5" t="n">
-        <v>12.30836772918701</v>
+        <v>11.55892086029053</v>
       </c>
     </row>
     <row r="6">
@@ -551,19 +551,19 @@
         <v>45839.16666666666</v>
       </c>
       <c r="B6" t="n">
-        <v>23.63061332702637</v>
+        <v>17.50858116149902</v>
       </c>
       <c r="C6" t="n">
-        <v>17.70819664001465</v>
+        <v>28.05973815917969</v>
       </c>
       <c r="D6" t="n">
-        <v>537.16015625</v>
+        <v>475.9024963378906</v>
       </c>
       <c r="E6" t="n">
-        <v>21.03122520446777</v>
+        <v>16.43264961242676</v>
       </c>
       <c r="F6" t="n">
-        <v>7.961918354034424</v>
+        <v>9.084312438964844</v>
       </c>
     </row>
     <row r="7">
@@ -571,19 +571,19 @@
         <v>45839.20833333334</v>
       </c>
       <c r="B7" t="n">
-        <v>20.58420944213867</v>
+        <v>22.99600219726562</v>
       </c>
       <c r="C7" t="n">
-        <v>39.04193878173828</v>
+        <v>31.42761611938477</v>
       </c>
       <c r="D7" t="n">
-        <v>820.4510498046875</v>
+        <v>814.5530395507812</v>
       </c>
       <c r="E7" t="n">
-        <v>24.30807495117188</v>
+        <v>16.69185829162598</v>
       </c>
       <c r="F7" t="n">
-        <v>9.540847778320312</v>
+        <v>7.99429178237915</v>
       </c>
     </row>
     <row r="8">
@@ -591,19 +591,19 @@
         <v>45839.25</v>
       </c>
       <c r="B8" t="n">
-        <v>19.79665756225586</v>
+        <v>28.96140670776367</v>
       </c>
       <c r="C8" t="n">
-        <v>56.87284088134766</v>
+        <v>27.80244445800781</v>
       </c>
       <c r="D8" t="n">
-        <v>1832.759887695312</v>
+        <v>1066.751220703125</v>
       </c>
       <c r="E8" t="n">
-        <v>21.9559383392334</v>
+        <v>22.12497520446777</v>
       </c>
       <c r="F8" t="n">
-        <v>6.762983322143555</v>
+        <v>11.93145751953125</v>
       </c>
     </row>
     <row r="9">
@@ -611,19 +611,19 @@
         <v>45839.29166666666</v>
       </c>
       <c r="B9" t="n">
-        <v>28.11669540405273</v>
+        <v>28.0385570526123</v>
       </c>
       <c r="C9" t="n">
-        <v>36.79299545288086</v>
+        <v>19.71765899658203</v>
       </c>
       <c r="D9" t="n">
-        <v>939.5449829101562</v>
+        <v>943.13720703125</v>
       </c>
       <c r="E9" t="n">
-        <v>36.57928848266602</v>
+        <v>31.32239151000977</v>
       </c>
       <c r="F9" t="n">
-        <v>5.515549182891846</v>
+        <v>13.73420715332031</v>
       </c>
     </row>
     <row r="10">
@@ -631,19 +631,19 @@
         <v>45839.33333333334</v>
       </c>
       <c r="B10" t="n">
-        <v>27.99954414367676</v>
+        <v>21.65900039672852</v>
       </c>
       <c r="C10" t="n">
-        <v>30.28523826599121</v>
+        <v>36.93322372436523</v>
       </c>
       <c r="D10" t="n">
-        <v>972.9308471679688</v>
+        <v>1416.498291015625</v>
       </c>
       <c r="E10" t="n">
-        <v>18.30448150634766</v>
+        <v>30.02301597595215</v>
       </c>
       <c r="F10" t="n">
-        <v>15.7487850189209</v>
+        <v>10.85761737823486</v>
       </c>
     </row>
     <row r="11">
@@ -651,19 +651,19 @@
         <v>45839.375</v>
       </c>
       <c r="B11" t="n">
-        <v>18.6532096862793</v>
+        <v>17.31425476074219</v>
       </c>
       <c r="C11" t="n">
-        <v>23.51878929138184</v>
+        <v>26.97262763977051</v>
       </c>
       <c r="D11" t="n">
-        <v>900.983642578125</v>
+        <v>646.0921020507812</v>
       </c>
       <c r="E11" t="n">
-        <v>27.44983863830566</v>
+        <v>17.1278018951416</v>
       </c>
       <c r="F11" t="n">
-        <v>10.78043746948242</v>
+        <v>13.49482536315918</v>
       </c>
     </row>
     <row r="12">
@@ -671,19 +671,19 @@
         <v>45839.41666666666</v>
       </c>
       <c r="B12" t="n">
-        <v>14.32156562805176</v>
+        <v>20.64898681640625</v>
       </c>
       <c r="C12" t="n">
-        <v>25.68955230712891</v>
+        <v>27.74266242980957</v>
       </c>
       <c r="D12" t="n">
-        <v>594.6871337890625</v>
+        <v>613.1823120117188</v>
       </c>
       <c r="E12" t="n">
-        <v>11.52461814880371</v>
+        <v>15.36508560180664</v>
       </c>
       <c r="F12" t="n">
-        <v>12.65956783294678</v>
+        <v>13.57704830169678</v>
       </c>
     </row>
     <row r="13">
@@ -691,19 +691,19 @@
         <v>45839.45833333334</v>
       </c>
       <c r="B13" t="n">
-        <v>26.8297061920166</v>
+        <v>21.04011535644531</v>
       </c>
       <c r="C13" t="n">
-        <v>24.3946533203125</v>
+        <v>30.5411491394043</v>
       </c>
       <c r="D13" t="n">
-        <v>399.4739074707031</v>
+        <v>461.1451110839844</v>
       </c>
       <c r="E13" t="n">
-        <v>12.52496433258057</v>
+        <v>13.18332195281982</v>
       </c>
       <c r="F13" t="n">
-        <v>16.97434425354004</v>
+        <v>17.85239601135254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(ai): re run notebooks after fixxing future covariates
</commit_message>
<xml_diff>
--- a/reports/nbeats_future_prediction_results.xlsx
+++ b/reports/nbeats_future_prediction_results.xlsx
@@ -471,19 +471,19 @@
         <v>45839</v>
       </c>
       <c r="B2" t="n">
-        <v>13.66680908203125</v>
+        <v>21.28914642333984</v>
       </c>
       <c r="C2" t="n">
-        <v>22.34885215759277</v>
+        <v>22.74205017089844</v>
       </c>
       <c r="D2" t="n">
-        <v>493.5171203613281</v>
+        <v>643.2750244140625</v>
       </c>
       <c r="E2" t="n">
-        <v>18.31430816650391</v>
+        <v>25.90433120727539</v>
       </c>
       <c r="F2" t="n">
-        <v>11.27921772003174</v>
+        <v>11.3208646774292</v>
       </c>
     </row>
     <row r="3">
@@ -491,19 +491,19 @@
         <v>45839.04166666666</v>
       </c>
       <c r="B3" t="n">
-        <v>15.72303199768066</v>
+        <v>17.26388740539551</v>
       </c>
       <c r="C3" t="n">
-        <v>21.53035163879395</v>
+        <v>21.13069725036621</v>
       </c>
       <c r="D3" t="n">
-        <v>480.7809143066406</v>
+        <v>734.884033203125</v>
       </c>
       <c r="E3" t="n">
-        <v>17.98626136779785</v>
+        <v>17.34470748901367</v>
       </c>
       <c r="F3" t="n">
-        <v>10.31490135192871</v>
+        <v>13.07268142700195</v>
       </c>
     </row>
     <row r="4">
@@ -511,19 +511,19 @@
         <v>45839.08333333334</v>
       </c>
       <c r="B4" t="n">
-        <v>13.92644500732422</v>
+        <v>20.79070663452148</v>
       </c>
       <c r="C4" t="n">
-        <v>20.73153495788574</v>
+        <v>29.03361129760742</v>
       </c>
       <c r="D4" t="n">
-        <v>393.5574951171875</v>
+        <v>764.6969604492188</v>
       </c>
       <c r="E4" t="n">
-        <v>22.21829223632812</v>
+        <v>23.04388427734375</v>
       </c>
       <c r="F4" t="n">
-        <v>6.941885948181152</v>
+        <v>9.320321083068848</v>
       </c>
     </row>
     <row r="5">
@@ -531,19 +531,19 @@
         <v>45839.125</v>
       </c>
       <c r="B5" t="n">
-        <v>19.11257553100586</v>
+        <v>17.59259223937988</v>
       </c>
       <c r="C5" t="n">
-        <v>28.15279197692871</v>
+        <v>23.69670295715332</v>
       </c>
       <c r="D5" t="n">
-        <v>570.4630126953125</v>
+        <v>456.4663391113281</v>
       </c>
       <c r="E5" t="n">
-        <v>21.31902503967285</v>
+        <v>18.03978157043457</v>
       </c>
       <c r="F5" t="n">
-        <v>11.55892086029053</v>
+        <v>12.30836772918701</v>
       </c>
     </row>
     <row r="6">
@@ -551,19 +551,19 @@
         <v>45839.16666666666</v>
       </c>
       <c r="B6" t="n">
-        <v>17.50858116149902</v>
+        <v>23.63061332702637</v>
       </c>
       <c r="C6" t="n">
-        <v>28.05973815917969</v>
+        <v>17.70819664001465</v>
       </c>
       <c r="D6" t="n">
-        <v>475.9024963378906</v>
+        <v>537.16015625</v>
       </c>
       <c r="E6" t="n">
-        <v>16.43264961242676</v>
+        <v>21.03122520446777</v>
       </c>
       <c r="F6" t="n">
-        <v>9.084312438964844</v>
+        <v>7.961918354034424</v>
       </c>
     </row>
     <row r="7">
@@ -571,19 +571,19 @@
         <v>45839.20833333334</v>
       </c>
       <c r="B7" t="n">
-        <v>22.99600219726562</v>
+        <v>20.58420944213867</v>
       </c>
       <c r="C7" t="n">
-        <v>31.42761611938477</v>
+        <v>39.04193878173828</v>
       </c>
       <c r="D7" t="n">
-        <v>814.5530395507812</v>
+        <v>820.4510498046875</v>
       </c>
       <c r="E7" t="n">
-        <v>16.69185829162598</v>
+        <v>24.30807495117188</v>
       </c>
       <c r="F7" t="n">
-        <v>7.99429178237915</v>
+        <v>9.540847778320312</v>
       </c>
     </row>
     <row r="8">
@@ -591,19 +591,19 @@
         <v>45839.25</v>
       </c>
       <c r="B8" t="n">
-        <v>28.96140670776367</v>
+        <v>19.79665756225586</v>
       </c>
       <c r="C8" t="n">
-        <v>27.80244445800781</v>
+        <v>56.87284088134766</v>
       </c>
       <c r="D8" t="n">
-        <v>1066.751220703125</v>
+        <v>1832.759887695312</v>
       </c>
       <c r="E8" t="n">
-        <v>22.12497520446777</v>
+        <v>21.9559383392334</v>
       </c>
       <c r="F8" t="n">
-        <v>11.93145751953125</v>
+        <v>6.762983322143555</v>
       </c>
     </row>
     <row r="9">
@@ -611,19 +611,19 @@
         <v>45839.29166666666</v>
       </c>
       <c r="B9" t="n">
-        <v>28.0385570526123</v>
+        <v>28.11669540405273</v>
       </c>
       <c r="C9" t="n">
-        <v>19.71765899658203</v>
+        <v>36.79299545288086</v>
       </c>
       <c r="D9" t="n">
-        <v>943.13720703125</v>
+        <v>939.5449829101562</v>
       </c>
       <c r="E9" t="n">
-        <v>31.32239151000977</v>
+        <v>36.57928848266602</v>
       </c>
       <c r="F9" t="n">
-        <v>13.73420715332031</v>
+        <v>5.515549182891846</v>
       </c>
     </row>
     <row r="10">
@@ -631,19 +631,19 @@
         <v>45839.33333333334</v>
       </c>
       <c r="B10" t="n">
-        <v>21.65900039672852</v>
+        <v>27.99954414367676</v>
       </c>
       <c r="C10" t="n">
-        <v>36.93322372436523</v>
+        <v>30.28523826599121</v>
       </c>
       <c r="D10" t="n">
-        <v>1416.498291015625</v>
+        <v>972.9308471679688</v>
       </c>
       <c r="E10" t="n">
-        <v>30.02301597595215</v>
+        <v>18.30448150634766</v>
       </c>
       <c r="F10" t="n">
-        <v>10.85761737823486</v>
+        <v>15.7487850189209</v>
       </c>
     </row>
     <row r="11">
@@ -651,19 +651,19 @@
         <v>45839.375</v>
       </c>
       <c r="B11" t="n">
-        <v>17.31425476074219</v>
+        <v>18.6532096862793</v>
       </c>
       <c r="C11" t="n">
-        <v>26.97262763977051</v>
+        <v>23.51878929138184</v>
       </c>
       <c r="D11" t="n">
-        <v>646.0921020507812</v>
+        <v>900.983642578125</v>
       </c>
       <c r="E11" t="n">
-        <v>17.1278018951416</v>
+        <v>27.44983863830566</v>
       </c>
       <c r="F11" t="n">
-        <v>13.49482536315918</v>
+        <v>10.78043746948242</v>
       </c>
     </row>
     <row r="12">
@@ -671,19 +671,19 @@
         <v>45839.41666666666</v>
       </c>
       <c r="B12" t="n">
-        <v>20.64898681640625</v>
+        <v>14.32156562805176</v>
       </c>
       <c r="C12" t="n">
-        <v>27.74266242980957</v>
+        <v>25.68955230712891</v>
       </c>
       <c r="D12" t="n">
-        <v>613.1823120117188</v>
+        <v>594.6871337890625</v>
       </c>
       <c r="E12" t="n">
-        <v>15.36508560180664</v>
+        <v>11.52461814880371</v>
       </c>
       <c r="F12" t="n">
-        <v>13.57704830169678</v>
+        <v>12.65956783294678</v>
       </c>
     </row>
     <row r="13">
@@ -691,19 +691,19 @@
         <v>45839.45833333334</v>
       </c>
       <c r="B13" t="n">
-        <v>21.04011535644531</v>
+        <v>26.8297061920166</v>
       </c>
       <c r="C13" t="n">
-        <v>30.5411491394043</v>
+        <v>24.3946533203125</v>
       </c>
       <c r="D13" t="n">
-        <v>461.1451110839844</v>
+        <v>399.4739074707031</v>
       </c>
       <c r="E13" t="n">
-        <v>13.18332195281982</v>
+        <v>12.52496433258057</v>
       </c>
       <c r="F13" t="n">
-        <v>17.85239601135254</v>
+        <v>16.97434425354004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>